<commit_message>
fix: dias_vencido es calculado, no campo de entrada
- Eliminado dias_vencido de cxc_aging.csv y plantilla_maestra.xlsx
- dias_vencido baja a campos_opcionales en cxc_aging_v1 (schema_registry)
- fecha_vencimiento es ahora el campo clave para calcular aging
- Removido dias_vencido de campos_recomendados en module_requirements:
  reporte_ejecutivo, kpi_cartera_cxc, vendedores_cxc
- Cards del panel actualizadas: nota visual explicando el calculo
- dias_vencido = hoy - fecha_vencimiento (calculado en tiempo real)
</commit_message>
<xml_diff>
--- a/templates/plantilla_maestra.xlsx
+++ b/templates/plantilla_maestra.xlsx
@@ -736,7 +736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -744,10 +744,9 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -778,20 +777,15 @@
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>dias_vencido</t>
+          <t>vendedor</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>vendedor</t>
+          <t>factura</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>factura</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>estatus</t>
         </is>
@@ -819,20 +813,17 @@
       <c r="E2" t="n">
         <v>30</v>
       </c>
-      <c r="F2" t="n">
-        <v>-11</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Carlos Méndez</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Carlos Méndez</t>
+          <t>F-1002</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
-        <is>
-          <t>F-1002</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
         <is>
           <t>Vigente</t>
         </is>
@@ -860,20 +851,17 @@
       <c r="E3" t="n">
         <v>30</v>
       </c>
-      <c r="F3" t="n">
-        <v>-25</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Ana López</t>
+        </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Ana López</t>
+          <t>F-1005</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
-        <is>
-          <t>F-1005</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
         <is>
           <t>Vigente</t>
         </is>
@@ -901,20 +889,17 @@
       <c r="E4" t="n">
         <v>30</v>
       </c>
-      <c r="F4" t="n">
-        <v>-30</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Carlos Méndez</t>
+        </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Carlos Méndez</t>
+          <t>F-1008</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
-        <is>
-          <t>F-1008</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
         <is>
           <t>Vigente</t>
         </is>
@@ -931,7 +916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -939,10 +924,9 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -973,20 +957,15 @@
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>dias_vencido</t>
+          <t>vendedor</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>vendedor</t>
+          <t>factura</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>factura</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>estatus</t>
         </is>
@@ -1014,20 +993,17 @@
       <c r="E2" t="n">
         <v>30</v>
       </c>
-      <c r="F2" t="n">
-        <v>109</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Ana López</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Ana López</t>
+          <t>F-1001</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
-        <is>
-          <t>F-1001</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
         <is>
           <t>Vencida</t>
         </is>
@@ -1055,20 +1031,17 @@
       <c r="E3" t="n">
         <v>30</v>
       </c>
-      <c r="F3" t="n">
-        <v>126</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Carlos Méndez</t>
+        </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Carlos Méndez</t>
+          <t>F-0990</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
-        <is>
-          <t>F-0990</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
         <is>
           <t>Vencida</t>
         </is>
@@ -1096,20 +1069,17 @@
       <c r="E4" t="n">
         <v>30</v>
       </c>
-      <c r="F4" t="n">
-        <v>171</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Ana López</t>
+        </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Ana López</t>
+          <t>F-0988</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
-        <is>
-          <t>F-0988</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
         <is>
           <t>Vencida</t>
         </is>
@@ -1137,20 +1107,17 @@
       <c r="E5" t="n">
         <v>30</v>
       </c>
-      <c r="F5" t="n">
-        <v>201</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Ana López</t>
+        </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Ana López</t>
+          <t>F-0950</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
-        <is>
-          <t>F-0950</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
         <is>
           <t>Vencida</t>
         </is>

</xml_diff>

<commit_message>
Revert "fix: dias_vencido es calculado, no campo de entrada"
This reverts commit c53007d1cfaae0bb69a88a523785b35a23b5d500.
</commit_message>
<xml_diff>
--- a/templates/plantilla_maestra.xlsx
+++ b/templates/plantilla_maestra.xlsx
@@ -736,7 +736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -744,9 +744,10 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -777,15 +778,20 @@
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
+          <t>dias_vencido</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
           <t>vendedor</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>factura</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>estatus</t>
         </is>
@@ -813,17 +819,20 @@
       <c r="E2" t="n">
         <v>30</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="n">
+        <v>-11</v>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Carlos Méndez</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>F-1002</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Vigente</t>
         </is>
@@ -851,17 +860,20 @@
       <c r="E3" t="n">
         <v>30</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" t="n">
+        <v>-25</v>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>Ana López</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>F-1005</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Vigente</t>
         </is>
@@ -889,17 +901,20 @@
       <c r="E4" t="n">
         <v>30</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" t="n">
+        <v>-30</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>Carlos Méndez</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>F-1008</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Vigente</t>
         </is>
@@ -916,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -924,9 +939,10 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -957,15 +973,20 @@
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
+          <t>dias_vencido</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
           <t>vendedor</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>factura</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>estatus</t>
         </is>
@@ -993,17 +1014,20 @@
       <c r="E2" t="n">
         <v>30</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="n">
+        <v>109</v>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Ana López</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>F-1001</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Vencida</t>
         </is>
@@ -1031,17 +1055,20 @@
       <c r="E3" t="n">
         <v>30</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" t="n">
+        <v>126</v>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>Carlos Méndez</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>F-0990</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Vencida</t>
         </is>
@@ -1069,17 +1096,20 @@
       <c r="E4" t="n">
         <v>30</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" t="n">
+        <v>171</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>Ana López</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>F-0988</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Vencida</t>
         </is>
@@ -1107,17 +1137,20 @@
       <c r="E5" t="n">
         <v>30</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" t="n">
+        <v>201</v>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>Ana López</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>F-0950</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Vencida</t>
         </is>

</xml_diff>

<commit_message>
fix(templates): quitar dias_vencido de plantillas CxC
dias_vencido es calculado por el sistema (hoy − fecha_vencimiento).
El usuario no debe proveerlo; solo necesita fecha_vencimiento.

Afecta:
- templates/cxc_aging.csv
- templates/plantilla_maestra.xlsx (hojas CXC VIGENTES y CXC VENCIDAS)
</commit_message>
<xml_diff>
--- a/templates/plantilla_maestra.xlsx
+++ b/templates/plantilla_maestra.xlsx
@@ -736,7 +736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -778,20 +778,15 @@
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>dias_vencido</t>
+          <t>vendedor</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>vendedor</t>
+          <t>factura</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>factura</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>estatus</t>
         </is>
@@ -819,20 +814,17 @@
       <c r="E2" t="n">
         <v>30</v>
       </c>
-      <c r="F2" t="n">
-        <v>-11</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Carlos Méndez</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Carlos Méndez</t>
+          <t>F-1002</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
-        <is>
-          <t>F-1002</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
         <is>
           <t>Vigente</t>
         </is>
@@ -860,20 +852,17 @@
       <c r="E3" t="n">
         <v>30</v>
       </c>
-      <c r="F3" t="n">
-        <v>-25</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Ana López</t>
+        </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Ana López</t>
+          <t>F-1005</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
-        <is>
-          <t>F-1005</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
         <is>
           <t>Vigente</t>
         </is>
@@ -901,20 +890,17 @@
       <c r="E4" t="n">
         <v>30</v>
       </c>
-      <c r="F4" t="n">
-        <v>-30</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Carlos Méndez</t>
+        </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Carlos Méndez</t>
+          <t>F-1008</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
-        <is>
-          <t>F-1008</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
         <is>
           <t>Vigente</t>
         </is>
@@ -931,7 +917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -973,20 +959,15 @@
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>dias_vencido</t>
+          <t>vendedor</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>vendedor</t>
+          <t>factura</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>factura</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>estatus</t>
         </is>
@@ -1014,20 +995,17 @@
       <c r="E2" t="n">
         <v>30</v>
       </c>
-      <c r="F2" t="n">
-        <v>109</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Ana López</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Ana López</t>
+          <t>F-1001</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
-        <is>
-          <t>F-1001</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
         <is>
           <t>Vencida</t>
         </is>
@@ -1055,20 +1033,17 @@
       <c r="E3" t="n">
         <v>30</v>
       </c>
-      <c r="F3" t="n">
-        <v>126</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Carlos Méndez</t>
+        </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Carlos Méndez</t>
+          <t>F-0990</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
-        <is>
-          <t>F-0990</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
         <is>
           <t>Vencida</t>
         </is>
@@ -1096,20 +1071,17 @@
       <c r="E4" t="n">
         <v>30</v>
       </c>
-      <c r="F4" t="n">
-        <v>171</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Ana López</t>
+        </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Ana López</t>
+          <t>F-0988</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
-        <is>
-          <t>F-0988</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
         <is>
           <t>Vencida</t>
         </is>
@@ -1137,20 +1109,17 @@
       <c r="E5" t="n">
         <v>30</v>
       </c>
-      <c r="F5" t="n">
-        <v>201</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Ana López</t>
+        </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Ana López</t>
+          <t>F-0950</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
-        <is>
-          <t>F-0950</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
         <is>
           <t>Vencida</t>
         </is>

</xml_diff>